<commit_message>
Add roster batted-ball radar chart to Rosters page
</commit_message>
<xml_diff>
--- a/data/dingers_player_data.xlsx
+++ b/data/dingers_player_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshbrodie/Desktop/claude_code/dingers/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C75687-1EFC-D844-A127-AC39027983AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4083E013-0051-D84D-A88A-542726E47F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="740" yWindow="1040" windowWidth="27240" windowHeight="16180" activeTab="2" xr2:uid="{60B155BA-D1AB-C646-8118-9D9B551D7988}"/>
+    <workbookView xWindow="720" yWindow="1040" windowWidth="27240" windowHeight="16180" activeTab="6" xr2:uid="{60B155BA-D1AB-C646-8118-9D9B551D7988}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,12 @@
     <sheet name="mlb_statcast" sheetId="3" r:id="rId3"/>
     <sheet name="games played" sheetId="2" r:id="rId4"/>
     <sheet name="team" sheetId="5" r:id="rId5"/>
+    <sheet name="injuries" sheetId="6" r:id="rId6"/>
+    <sheet name="team_stats" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'games played'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">injuries!$A$1:$F$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MAIN!$A$1:$I$500</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6218" uniqueCount="2227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6595" uniqueCount="2307">
   <si>
     <t>Rk</t>
   </si>
@@ -6722,13 +6725,253 @@
   </si>
   <si>
     <t>mlb_statcast_name</t>
+  </si>
+  <si>
+    <t>Injury / Surgery</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Latest Update</t>
+  </si>
+  <si>
+    <t>60-Day IL</t>
+  </si>
+  <si>
+    <t>No timetable for return</t>
+  </si>
+  <si>
+    <t>Shoulder surgery (torn labrum)</t>
+  </si>
+  <si>
+    <t>Rehab assignment (6/30)</t>
+  </si>
+  <si>
+    <t>Rehab assignment (7/12)</t>
+  </si>
+  <si>
+    <t>Questionable for 2026 season</t>
+  </si>
+  <si>
+    <t>Out for 2026 season</t>
+  </si>
+  <si>
+    <t>Arthroscopic knee surgery</t>
+  </si>
+  <si>
+    <t>Bone bruise in foot</t>
+  </si>
+  <si>
+    <t>Strained calf</t>
+  </si>
+  <si>
+    <t>10-Day IL</t>
+  </si>
+  <si>
+    <t>Dislocated shoulder</t>
+  </si>
+  <si>
+    <t>Expected to miss 4-6 months</t>
+  </si>
+  <si>
+    <t>Lumbar spine disc herniation</t>
+  </si>
+  <si>
+    <t>Sprained ankle</t>
+  </si>
+  <si>
+    <t>Fractured thumb (left)</t>
+  </si>
+  <si>
+    <t>Elbow lateral epicondylitis (right)</t>
+  </si>
+  <si>
+    <t>Sprained finger (right ring)</t>
+  </si>
+  <si>
+    <t>Elbow inflammation</t>
+  </si>
+  <si>
+    <t>Plantar fasciitis</t>
+  </si>
+  <si>
+    <t>Ankle surgery (torn tendon)</t>
+  </si>
+  <si>
+    <t>Strained groin</t>
+  </si>
+  <si>
+    <t>Hernia</t>
+  </si>
+  <si>
+    <t>Knee inflammation</t>
+  </si>
+  <si>
+    <t>Oblique contusion</t>
+  </si>
+  <si>
+    <t>Sports hernia surgery</t>
+  </si>
+  <si>
+    <t>Expected to miss 6-10 weeks</t>
+  </si>
+  <si>
+    <t>Rehab assignment (7/13)</t>
+  </si>
+  <si>
+    <t>Sprained elbow</t>
+  </si>
+  <si>
+    <t>Strained oblique</t>
+  </si>
+  <si>
+    <t>Wrist contusion</t>
+  </si>
+  <si>
+    <t>Rehab assignment (6/22)</t>
+  </si>
+  <si>
+    <t>Heel discomfort</t>
+  </si>
+  <si>
+    <t>Fractured hand</t>
+  </si>
+  <si>
+    <t>Rib stress fracture</t>
+  </si>
+  <si>
+    <t>Will be re-evaluated in 4-6 weeks</t>
+  </si>
+  <si>
+    <t>Strained hamstring</t>
+  </si>
+  <si>
+    <t>Neck inflammation</t>
+  </si>
+  <si>
+    <t>Hip surgery (torn labrum)</t>
+  </si>
+  <si>
+    <t>Fourth and fifth metacarpal fractures</t>
+  </si>
+  <si>
+    <t>Expected to miss 4-6 weeks</t>
+  </si>
+  <si>
+    <t>Fractured hamate (left hand)</t>
+  </si>
+  <si>
+    <t>Expected to miss at least 4 weeks</t>
+  </si>
+  <si>
+    <t>Non-displaced fracture (foot)</t>
+  </si>
+  <si>
+    <t>Hamate surgery (left hand)</t>
+  </si>
+  <si>
+    <t>Expected to miss 5-7 weeks</t>
+  </si>
+  <si>
+    <t>Orbital fracture</t>
+  </si>
+  <si>
+    <t>Strained hand (left)</t>
+  </si>
+  <si>
+    <t>Concussion</t>
+  </si>
+  <si>
+    <t>7-Day IL</t>
+  </si>
+  <si>
+    <t>Forearm inflammation</t>
+  </si>
+  <si>
+    <t>Strained glute</t>
+  </si>
+  <si>
+    <t>Rehab assignment (7/9)</t>
+  </si>
+  <si>
+    <t>Strained hip flexor</t>
+  </si>
+  <si>
+    <t>Lat surgery</t>
+  </si>
+  <si>
+    <t>Stress reaction in forearm</t>
+  </si>
+  <si>
+    <t>Strained lower back</t>
+  </si>
+  <si>
+    <t>Sprained hand (left)</t>
+  </si>
+  <si>
+    <t>Shoulder contusion</t>
+  </si>
+  <si>
+    <t>Finger inflammation (right middle)</t>
+  </si>
+  <si>
+    <t>Strained abdominal</t>
+  </si>
+  <si>
+    <t>Lower back inflammation</t>
+  </si>
+  <si>
+    <t>Knee surgery</t>
+  </si>
+  <si>
+    <t>Head contusion</t>
+  </si>
+  <si>
+    <t>Rehab assignment (7/8)</t>
+  </si>
+  <si>
+    <t>Strained hip</t>
+  </si>
+  <si>
+    <t>Torn finger tendon (left ring)</t>
+  </si>
+  <si>
+    <t>Expected to miss 8-10 weeks</t>
+  </si>
+  <si>
+    <t>Knee laceration</t>
+  </si>
+  <si>
+    <t>Sprained thumb capsule</t>
+  </si>
+  <si>
+    <t>Fractured hand (right)</t>
+  </si>
+  <si>
+    <t>Elbow inflammation (non-throwing)</t>
+  </si>
+  <si>
+    <t>Match Name</t>
+  </si>
+  <si>
+    <t>Player ID</t>
+  </si>
+  <si>
+    <t>exp_home_run</t>
+  </si>
+  <si>
+    <t>hr_per_4_pa</t>
+  </si>
+  <si>
+    <t>no_doubter_per</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -6919,6 +7162,30 @@
     <font>
       <sz val="10.199999999999999"/>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -7263,7 +7530,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -7293,6 +7560,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -23680,6 +23952,7 @@
   </sheetData>
   <autoFilter ref="A1:I500" xr:uid="{438BCB09-DCEC-4A42-812B-1E04B50EE495}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -89942,4 +90215,4281 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE878EF0-8C69-0048-AFB3-3CF2536C7408}">
+  <dimension ref="A1:F68"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>514</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>2302</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>2303</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>2228</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>2227</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>2229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B2" t="str">
+        <f>_xlfn.XLOOKUP($A2,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Denzel Clarke</v>
+      </c>
+      <c r="C2">
+        <f>_xlfn.XLOOKUP($B2,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>672016</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>2238</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" t="str">
+        <f>_xlfn.XLOOKUP($A3,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Giancarlo Stanton</v>
+      </c>
+      <c r="C3">
+        <f>_xlfn.XLOOKUP($B3,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>519317</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>2239</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B4" t="str">
+        <f>_xlfn.XLOOKUP($A4,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Tanner Murray</v>
+      </c>
+      <c r="C4">
+        <f>_xlfn.XLOOKUP($B4,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>695020</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>2241</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B5" t="str">
+        <f>_xlfn.XLOOKUP($A5,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Luis Robert Jr.</v>
+      </c>
+      <c r="C5">
+        <f>_xlfn.XLOOKUP($B5,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>673357</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>2243</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>2233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6" t="str">
+        <f>_xlfn.XLOOKUP($A6,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Javier Báez</v>
+      </c>
+      <c r="C6">
+        <f>_xlfn.XLOOKUP($B6,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>595879</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>2244</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" t="str">
+        <f>_xlfn.XLOOKUP($A7,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Jonathan India</v>
+      </c>
+      <c r="C7">
+        <f>_xlfn.XLOOKUP($B7,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>663697</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>2232</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>260</v>
+      </c>
+      <c r="B8" t="str">
+        <f>_xlfn.XLOOKUP($A8,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Will Wilson</v>
+      </c>
+      <c r="C8">
+        <f>_xlfn.XLOOKUP($B8,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>669717</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>2245</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B9" t="str">
+        <f>_xlfn.XLOOKUP($A9,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Austin Hays</v>
+      </c>
+      <c r="C9">
+        <f>_xlfn.XLOOKUP($B9,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>669720</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>2239</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10" t="str">
+        <f>_xlfn.XLOOKUP($A10,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Ramón Urías</v>
+      </c>
+      <c r="C10">
+        <f>_xlfn.XLOOKUP($B10,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>602104</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>2246</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>439</v>
+      </c>
+      <c r="B11" t="str">
+        <f>_xlfn.XLOOKUP($A11,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Roman Anthony</v>
+      </c>
+      <c r="C11">
+        <f>_xlfn.XLOOKUP($B11,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>701350</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>2247</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>248</v>
+      </c>
+      <c r="B12" t="str">
+        <f>_xlfn.XLOOKUP($A12,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Travis d'Arnaud</v>
+      </c>
+      <c r="C12">
+        <f>_xlfn.XLOOKUP($B12,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>518595</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>2249</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" t="str">
+        <f>_xlfn.XLOOKUP($A13,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Carlos Correa</v>
+      </c>
+      <c r="C13">
+        <f>_xlfn.XLOOKUP($B13,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>621043</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>2250</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>413</v>
+      </c>
+      <c r="B14" t="str">
+        <f>_xlfn.XLOOKUP($A14,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Brendan Donovan</v>
+      </c>
+      <c r="C14">
+        <f>_xlfn.XLOOKUP($B14,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>680977</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>2251</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>426</v>
+      </c>
+      <c r="B15" t="str">
+        <f>_xlfn.XLOOKUP($A15,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Jake Fraley</v>
+      </c>
+      <c r="C15">
+        <f>_xlfn.XLOOKUP($B15,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>641584</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>2252</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" t="str">
+        <f>_xlfn.XLOOKUP($A16,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Brenton Doyle</v>
+      </c>
+      <c r="C16">
+        <f>_xlfn.XLOOKUP($B16,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>686668</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>2254</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>490</v>
+      </c>
+      <c r="B17" t="str">
+        <f>_xlfn.XLOOKUP($A17,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Yoán Moncada</v>
+      </c>
+      <c r="C17">
+        <f>_xlfn.XLOOKUP($B17,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>660162</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>2253</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>172</v>
+      </c>
+      <c r="B18" t="str">
+        <f>_xlfn.XLOOKUP($A18,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Trevor Story</v>
+      </c>
+      <c r="C18">
+        <f>_xlfn.XLOOKUP($B18,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>596115</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>2255</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>2256</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B19" t="str">
+        <f>_xlfn.XLOOKUP($A19,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Enrique Hernández</v>
+      </c>
+      <c r="C19">
+        <f>_xlfn.XLOOKUP($B19,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>571771</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>2259</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" t="str">
+        <f>_xlfn.XLOOKUP($A20,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Lenyn Sosa</v>
+      </c>
+      <c r="C20">
+        <f>_xlfn.XLOOKUP($B20,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>672820</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>2260</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>135</v>
+      </c>
+      <c r="B21" t="str">
+        <f>_xlfn.XLOOKUP($A21,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Harrison Bader</v>
+      </c>
+      <c r="C21">
+        <f>_xlfn.XLOOKUP($B21,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>664056</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>2262</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" t="str">
+        <f>_xlfn.XLOOKUP($A22,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Aaron Judge</v>
+      </c>
+      <c r="C22">
+        <f>_xlfn.XLOOKUP($B22,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>592450</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>2264</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>2265</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>444</v>
+      </c>
+      <c r="B23" t="str">
+        <f>_xlfn.XLOOKUP($A23,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Adam Frazier</v>
+      </c>
+      <c r="C23">
+        <f>_xlfn.XLOOKUP($B23,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>624428</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>2248</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" t="str">
+        <f>_xlfn.XLOOKUP($A24,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Will Smith</v>
+      </c>
+      <c r="C24">
+        <f>_xlfn.XLOOKUP($B24,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>669257</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>2267</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" t="str">
+        <f>_xlfn.XLOOKUP($A25,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Ramón Laureano</v>
+      </c>
+      <c r="C25">
+        <f>_xlfn.XLOOKUP($B25,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>657656</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>2268</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>311</v>
+      </c>
+      <c r="B26" t="str">
+        <f>_xlfn.XLOOKUP($A26,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Oneil Cruz</v>
+      </c>
+      <c r="C26">
+        <f>_xlfn.XLOOKUP($B26,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>665833</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>2269</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>101</v>
+      </c>
+      <c r="B27" t="str">
+        <f>_xlfn.XLOOKUP($A27,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Ronald Acuña Jr.</v>
+      </c>
+      <c r="C27">
+        <f>_xlfn.XLOOKUP($B27,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>660670</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>2266</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>407</v>
+      </c>
+      <c r="B28" t="str">
+        <f>_xlfn.XLOOKUP($A28,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Kyle Isbel</v>
+      </c>
+      <c r="C28">
+        <f>_xlfn.XLOOKUP($B28,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>664728</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>2249</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>272</v>
+      </c>
+      <c r="B29" t="str">
+        <f>_xlfn.XLOOKUP($A29,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Sebastián Rivero</v>
+      </c>
+      <c r="C29">
+        <f>_xlfn.XLOOKUP($B29,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>665861</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>2271</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>2272</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>467</v>
+      </c>
+      <c r="B30" t="str">
+        <f>_xlfn.XLOOKUP($A30,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Angel Martínez</v>
+      </c>
+      <c r="C30">
+        <f>_xlfn.XLOOKUP($B30,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>682657</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>2273</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>251</v>
+      </c>
+      <c r="B31" t="str">
+        <f>_xlfn.XLOOKUP($A31,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Michael Helman</v>
+      </c>
+      <c r="C31">
+        <f>_xlfn.XLOOKUP($B31,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>680737</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>2263</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>147</v>
+      </c>
+      <c r="B32" t="str">
+        <f>_xlfn.XLOOKUP($A32,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Gleyber Torres</v>
+      </c>
+      <c r="C32">
+        <f>_xlfn.XLOOKUP($B32,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>650402</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>2259</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>468</v>
+      </c>
+      <c r="B33" t="str">
+        <f>_xlfn.XLOOKUP($A33,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>José Ramírez</v>
+      </c>
+      <c r="C33">
+        <f>_xlfn.XLOOKUP($B33,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>608070</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>2274</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>2275</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>478</v>
+      </c>
+      <c r="B34" t="str">
+        <f>_xlfn.XLOOKUP($A34,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Wenceel Pérez</v>
+      </c>
+      <c r="C34">
+        <f>_xlfn.XLOOKUP($B34,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>672761</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" t="str">
+        <f>_xlfn.XLOOKUP($A35,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Maikel Garcia</v>
+      </c>
+      <c r="C35">
+        <f>_xlfn.XLOOKUP($B35,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>672580</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>2277</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" t="str">
+        <f>_xlfn.XLOOKUP($A36,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Everson Pereira</v>
+      </c>
+      <c r="C36">
+        <f>_xlfn.XLOOKUP($B36,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>677592</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>2278</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>199</v>
+      </c>
+      <c r="B37" t="str">
+        <f>_xlfn.XLOOKUP($A37,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Isiah Kiner-Falefa</v>
+      </c>
+      <c r="C37">
+        <f>_xlfn.XLOOKUP($B37,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>643396</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>2280</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>245</v>
+      </c>
+      <c r="B38" t="str">
+        <f>_xlfn.XLOOKUP($A38,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Jordan Lawlar</v>
+      </c>
+      <c r="C38">
+        <f>_xlfn.XLOOKUP($B38,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>691783</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>2266</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>265</v>
+      </c>
+      <c r="B39" t="str">
+        <f>_xlfn.XLOOKUP($A39,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Brandon Lockridge</v>
+      </c>
+      <c r="C39">
+        <f>_xlfn.XLOOKUP($B39,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>663604</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>2237</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" t="str">
+        <f>_xlfn.XLOOKUP($A40,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Marcus Semien</v>
+      </c>
+      <c r="C40">
+        <f>_xlfn.XLOOKUP($B40,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>543760</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>2283</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" t="str">
+        <f>_xlfn.XLOOKUP($A41,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Adolis García</v>
+      </c>
+      <c r="C41">
+        <f>_xlfn.XLOOKUP($B41,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>666969</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>2284</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>337</v>
+      </c>
+      <c r="B42" t="str">
+        <f>_xlfn.XLOOKUP($A42,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Spencer Horwitz</v>
+      </c>
+      <c r="C42">
+        <f>_xlfn.XLOOKUP($B42,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>687462</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>2266</v>
+      </c>
+      <c r="F42" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>402</v>
+      </c>
+      <c r="B43" t="str">
+        <f>_xlfn.XLOOKUP($A43,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Marcelo Mayer</v>
+      </c>
+      <c r="C43">
+        <f>_xlfn.XLOOKUP($B43,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>691785</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E43" s="14" t="s">
+        <v>2285</v>
+      </c>
+      <c r="F43" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>263</v>
+      </c>
+      <c r="B44" t="str">
+        <f>_xlfn.XLOOKUP($A44,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Daniel Susac</v>
+      </c>
+      <c r="C44">
+        <f>_xlfn.XLOOKUP($B44,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>691740</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>2286</v>
+      </c>
+      <c r="F44" s="14" t="s">
+        <v>2282</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>197</v>
+      </c>
+      <c r="B45" t="str">
+        <f>_xlfn.XLOOKUP($A45,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Blake Dunn</v>
+      </c>
+      <c r="C45">
+        <f>_xlfn.XLOOKUP($B45,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>694362</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>2258</v>
+      </c>
+      <c r="F45" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>182</v>
+      </c>
+      <c r="B46" t="str">
+        <f>_xlfn.XLOOKUP($A46,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Rob Refsnyder</v>
+      </c>
+      <c r="C46">
+        <f>_xlfn.XLOOKUP($B46,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>608701</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>2253</v>
+      </c>
+      <c r="F46" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>361</v>
+      </c>
+      <c r="B47" t="str">
+        <f>_xlfn.XLOOKUP($A47,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Jesús Sánchez</v>
+      </c>
+      <c r="C47">
+        <f>_xlfn.XLOOKUP($B47,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>660821</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>2244</v>
+      </c>
+      <c r="F47" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>151</v>
+      </c>
+      <c r="B48" t="str">
+        <f>_xlfn.XLOOKUP($A48,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Matt Shaw</v>
+      </c>
+      <c r="C48">
+        <f>_xlfn.XLOOKUP($B48,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>807713</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>2287</v>
+      </c>
+      <c r="F48" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>181</v>
+      </c>
+      <c r="B49" t="str">
+        <f>_xlfn.XLOOKUP($A49,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Dane Myers</v>
+      </c>
+      <c r="C49">
+        <f>_xlfn.XLOOKUP($B49,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>667472</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>2288</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>267</v>
+      </c>
+      <c r="B50" t="str">
+        <f>_xlfn.XLOOKUP($A50,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Ha-Seong Kim</v>
+      </c>
+      <c r="C50">
+        <f>_xlfn.XLOOKUP($B50,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>673490</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>2289</v>
+      </c>
+      <c r="F50" s="14" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>96</v>
+      </c>
+      <c r="B51" t="str">
+        <f>_xlfn.XLOOKUP($A51,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Matt Chapman</v>
+      </c>
+      <c r="C51">
+        <f>_xlfn.XLOOKUP($B51,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>656305</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>2290</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>340</v>
+      </c>
+      <c r="B52" t="str">
+        <f>_xlfn.XLOOKUP($A52,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Corey Seager</v>
+      </c>
+      <c r="C52">
+        <f>_xlfn.XLOOKUP($B52,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>608369</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>2291</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53" t="str">
+        <f>_xlfn.XLOOKUP($A53,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Brent Rooker</v>
+      </c>
+      <c r="C53">
+        <f>_xlfn.XLOOKUP($B53,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>667670</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>2292</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>174</v>
+      </c>
+      <c r="B54" t="str">
+        <f>_xlfn.XLOOKUP($A54,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Freddy Fermin</v>
+      </c>
+      <c r="C54">
+        <f>_xlfn.XLOOKUP($B54,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>666023</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>2293</v>
+      </c>
+      <c r="F54" s="14" t="s">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>40</v>
+      </c>
+      <c r="B55" t="str">
+        <f>_xlfn.XLOOKUP($A55,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Julio Rodríguez</v>
+      </c>
+      <c r="C55">
+        <f>_xlfn.XLOOKUP($B55,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>677594</v>
+      </c>
+      <c r="D55" s="14" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>2278</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>10</v>
+      </c>
+      <c r="B56" t="str">
+        <f>_xlfn.XLOOKUP($A56,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Byron Buxton</v>
+      </c>
+      <c r="C56">
+        <f>_xlfn.XLOOKUP($B56,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>621439</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>2295</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>484</v>
+      </c>
+      <c r="B57" t="str">
+        <f>_xlfn.XLOOKUP($A57,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Endy Rodríguez</v>
+      </c>
+      <c r="C57">
+        <f>_xlfn.XLOOKUP($B57,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>682848</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E57" s="14" t="s">
+        <v>2281</v>
+      </c>
+      <c r="F57" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>253</v>
+      </c>
+      <c r="B58" t="str">
+        <f>_xlfn.XLOOKUP($A58,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Jonah Cox</v>
+      </c>
+      <c r="C58">
+        <f>_xlfn.XLOOKUP($B58,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>813841</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E58" s="14" t="s">
+        <v>2259</v>
+      </c>
+      <c r="F58" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>401</v>
+      </c>
+      <c r="B59" t="str">
+        <f>_xlfn.XLOOKUP($A59,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>David Hamilton</v>
+      </c>
+      <c r="C59">
+        <f>_xlfn.XLOOKUP($B59,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>666152</v>
+      </c>
+      <c r="D59" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E59" s="14" t="s">
+        <v>2266</v>
+      </c>
+      <c r="F59" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>126</v>
+      </c>
+      <c r="B60" t="str">
+        <f>_xlfn.XLOOKUP($A60,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Konnor Griffin</v>
+      </c>
+      <c r="C60">
+        <f>_xlfn.XLOOKUP($B60,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>804606</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E60" s="14" t="s">
+        <v>2296</v>
+      </c>
+      <c r="F60" s="14" t="s">
+        <v>2297</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61" t="str">
+        <f>_xlfn.XLOOKUP($A61,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Matt McLain</v>
+      </c>
+      <c r="C61">
+        <f>_xlfn.XLOOKUP($B61,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>680574</v>
+      </c>
+      <c r="D61" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E61" s="14" t="s">
+        <v>2239</v>
+      </c>
+      <c r="F61" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>228</v>
+      </c>
+      <c r="B62" t="str">
+        <f>_xlfn.XLOOKUP($A62,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Samad Taylor</v>
+      </c>
+      <c r="C62">
+        <f>_xlfn.XLOOKUP($B62,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>669392</v>
+      </c>
+      <c r="D62" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E62" s="14" t="s">
+        <v>2259</v>
+      </c>
+      <c r="F62" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>323</v>
+      </c>
+      <c r="B63" t="str">
+        <f>_xlfn.XLOOKUP($A63,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Owen Caissie</v>
+      </c>
+      <c r="C63">
+        <f>_xlfn.XLOOKUP($B63,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>683357</v>
+      </c>
+      <c r="D63" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E63" s="14" t="s">
+        <v>2239</v>
+      </c>
+      <c r="F63" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64" t="str">
+        <f>_xlfn.XLOOKUP($A64,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Zack Gelof</v>
+      </c>
+      <c r="C64">
+        <f>_xlfn.XLOOKUP($B64,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>680869</v>
+      </c>
+      <c r="D64" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E64" s="14" t="s">
+        <v>2298</v>
+      </c>
+      <c r="F64" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>286</v>
+      </c>
+      <c r="B65" t="str">
+        <f>_xlfn.XLOOKUP($A65,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Nick Kurtz</v>
+      </c>
+      <c r="C65">
+        <f>_xlfn.XLOOKUP($B65,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>701762</v>
+      </c>
+      <c r="D65" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E65" s="14" t="s">
+        <v>2299</v>
+      </c>
+      <c r="F65" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>59</v>
+      </c>
+      <c r="B66" t="str">
+        <f>_xlfn.XLOOKUP($A66,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Mark Vientos</v>
+      </c>
+      <c r="C66">
+        <f>_xlfn.XLOOKUP($B66,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>668901</v>
+      </c>
+      <c r="D66" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E66" s="14" t="s">
+        <v>2300</v>
+      </c>
+      <c r="F66" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>531</v>
+      </c>
+      <c r="B67" t="str">
+        <f>_xlfn.XLOOKUP($A67,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Victor Bericoto</v>
+      </c>
+      <c r="C67">
+        <f>_xlfn.XLOOKUP($B67,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>682674</v>
+      </c>
+      <c r="D67" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E67" s="14" t="s">
+        <v>2259</v>
+      </c>
+      <c r="F67" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>371</v>
+      </c>
+      <c r="B68" t="str">
+        <f>_xlfn.XLOOKUP($A68,MAIN!C:C,MAIN!C:C,"xxx")</f>
+        <v>Mike Yastrzemski</v>
+      </c>
+      <c r="C68">
+        <f>_xlfn.XLOOKUP($B68,MAIN!$C:$C,MAIN!$B:$B,"xxx")</f>
+        <v>573262</v>
+      </c>
+      <c r="D68" s="14" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E68" s="14" t="s">
+        <v>2301</v>
+      </c>
+      <c r="F68" s="14" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F68" xr:uid="{BE878EF0-8C69-0048-AFB3-3CF2536C7408}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6B2B3E9-7332-1E40-9045-0257B743AEA0}">
+  <dimension ref="A1:I95"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>693</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>2304</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>2305</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>698</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>700</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>2306</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>699</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="16">
+        <v>691023</v>
+      </c>
+      <c r="C2" s="16">
+        <v>20.5</v>
+      </c>
+      <c r="D2" s="16">
+        <v>0.22</v>
+      </c>
+      <c r="E2" s="16">
+        <v>79.2</v>
+      </c>
+      <c r="F2" s="16">
+        <v>11.5</v>
+      </c>
+      <c r="G2" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="H2" s="16">
+        <v>94.2</v>
+      </c>
+      <c r="I2" s="17">
+        <v>0.14099999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="16">
+        <v>624413</v>
+      </c>
+      <c r="C3" s="16">
+        <v>20.8</v>
+      </c>
+      <c r="D3" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E3" s="16">
+        <v>74.8</v>
+      </c>
+      <c r="F3" s="16">
+        <v>14.4</v>
+      </c>
+      <c r="G3" s="17">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="H3" s="16">
+        <v>93.8</v>
+      </c>
+      <c r="I3" s="17">
+        <v>0.126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" s="16">
+        <v>701762</v>
+      </c>
+      <c r="C4" s="16">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="D4" s="16">
+        <v>0.19</v>
+      </c>
+      <c r="E4" s="16">
+        <v>78.3</v>
+      </c>
+      <c r="F4" s="16">
+        <v>12.4</v>
+      </c>
+      <c r="G4" s="17">
+        <v>0.4</v>
+      </c>
+      <c r="H4" s="16">
+        <v>93.6</v>
+      </c>
+      <c r="I4" s="17">
+        <v>0.18099999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="16">
+        <v>669127</v>
+      </c>
+      <c r="C5" s="16">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="D5" s="16">
+        <v>0.22</v>
+      </c>
+      <c r="E5" s="16">
+        <v>75.2</v>
+      </c>
+      <c r="F5" s="16">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="G5" s="17">
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="H5" s="16">
+        <v>91.8</v>
+      </c>
+      <c r="I5" s="17">
+        <v>0.14699999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="B6" s="16">
+        <v>656941</v>
+      </c>
+      <c r="C6" s="16">
+        <v>28</v>
+      </c>
+      <c r="D6" s="16">
+        <v>0.31</v>
+      </c>
+      <c r="E6" s="16">
+        <v>77.099999999999994</v>
+      </c>
+      <c r="F6" s="16">
+        <v>21.8</v>
+      </c>
+      <c r="G6" s="17">
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="H6" s="16">
+        <v>93.4</v>
+      </c>
+      <c r="I6" s="17">
+        <v>0.19400000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="16" t="s">
+        <v>469</v>
+      </c>
+      <c r="B7" s="16">
+        <v>663728</v>
+      </c>
+      <c r="C7" s="16">
+        <v>11.1</v>
+      </c>
+      <c r="D7" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E7" s="16">
+        <v>74.7</v>
+      </c>
+      <c r="F7" s="16">
+        <v>24</v>
+      </c>
+      <c r="G7" s="17">
+        <v>0.55600000000000005</v>
+      </c>
+      <c r="H7" s="16">
+        <v>88.2</v>
+      </c>
+      <c r="I7" s="17">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="16" t="s">
+        <v>281</v>
+      </c>
+      <c r="B8" s="16">
+        <v>695657</v>
+      </c>
+      <c r="C8" s="16">
+        <v>23.1</v>
+      </c>
+      <c r="D8" s="16">
+        <v>0.24</v>
+      </c>
+      <c r="E8" s="16">
+        <v>76.3</v>
+      </c>
+      <c r="F8" s="16">
+        <v>23</v>
+      </c>
+      <c r="G8" s="17">
+        <v>0.47799999999999998</v>
+      </c>
+      <c r="H8" s="16">
+        <v>89.2</v>
+      </c>
+      <c r="I8" s="17">
+        <v>0.13700000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="16" t="s">
+        <v>278</v>
+      </c>
+      <c r="B9" s="16">
+        <v>700250</v>
+      </c>
+      <c r="C9" s="16">
+        <v>27.5</v>
+      </c>
+      <c r="D9" s="16">
+        <v>0.3</v>
+      </c>
+      <c r="E9" s="16">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="F9" s="16">
+        <v>14.2</v>
+      </c>
+      <c r="G9" s="17">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="H9" s="16">
+        <v>92.1</v>
+      </c>
+      <c r="I9" s="17">
+        <v>0.153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="B10" s="16">
+        <v>670541</v>
+      </c>
+      <c r="C10" s="16">
+        <v>35.299999999999997</v>
+      </c>
+      <c r="D10" s="16">
+        <v>0.3</v>
+      </c>
+      <c r="E10" s="16">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="F10" s="16">
+        <v>19.8</v>
+      </c>
+      <c r="G10" s="17">
+        <v>0.61299999999999999</v>
+      </c>
+      <c r="H10" s="16">
+        <v>94.7</v>
+      </c>
+      <c r="I10" s="17">
+        <v>0.187</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="16">
+        <v>696100</v>
+      </c>
+      <c r="C11" s="16">
+        <v>22</v>
+      </c>
+      <c r="D11" s="16">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="E11" s="16">
+        <v>75.3</v>
+      </c>
+      <c r="F11" s="16">
+        <v>18</v>
+      </c>
+      <c r="G11" s="17">
+        <v>0.51900000000000002</v>
+      </c>
+      <c r="H11" s="16">
+        <v>91.2</v>
+      </c>
+      <c r="I11" s="17">
+        <v>0.16600000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="16">
+        <v>691406</v>
+      </c>
+      <c r="C12" s="16">
+        <v>26</v>
+      </c>
+      <c r="D12" s="16">
+        <v>0.27</v>
+      </c>
+      <c r="E12" s="16">
+        <v>79.900000000000006</v>
+      </c>
+      <c r="F12" s="16">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="G12" s="17">
+        <v>0.67900000000000005</v>
+      </c>
+      <c r="H12" s="16">
+        <v>93.2</v>
+      </c>
+      <c r="I12" s="17">
+        <v>0.13600000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="16">
+        <v>621439</v>
+      </c>
+      <c r="C13" s="16">
+        <v>26</v>
+      </c>
+      <c r="D13" s="16">
+        <v>0.3</v>
+      </c>
+      <c r="E13" s="16">
+        <v>74.2</v>
+      </c>
+      <c r="F13" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="G13" s="17">
+        <v>0.52</v>
+      </c>
+      <c r="H13" s="16">
+        <v>90.7</v>
+      </c>
+      <c r="I13" s="17">
+        <v>0.187</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" s="16">
+        <v>671277</v>
+      </c>
+      <c r="C14" s="16">
+        <v>17.7</v>
+      </c>
+      <c r="D14" s="16">
+        <v>0.25</v>
+      </c>
+      <c r="E14" s="16">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="F14" s="16">
+        <v>11.5</v>
+      </c>
+      <c r="G14" s="17">
+        <v>0.35</v>
+      </c>
+      <c r="H14" s="16">
+        <v>91.9</v>
+      </c>
+      <c r="I14" s="17">
+        <v>0.107</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="B15" s="16">
+        <v>665742</v>
+      </c>
+      <c r="C15" s="16">
+        <v>22.5</v>
+      </c>
+      <c r="D15" s="16">
+        <v>0.25</v>
+      </c>
+      <c r="E15" s="16">
+        <v>72</v>
+      </c>
+      <c r="F15" s="16">
+        <v>15.9</v>
+      </c>
+      <c r="G15" s="17">
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="H15" s="16">
+        <v>92.6</v>
+      </c>
+      <c r="I15" s="17">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="16">
+        <v>687263</v>
+      </c>
+      <c r="C16" s="16">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="D16" s="16">
+        <v>0.18</v>
+      </c>
+      <c r="E16" s="16">
+        <v>71</v>
+      </c>
+      <c r="F16" s="16">
+        <v>22.1</v>
+      </c>
+      <c r="G16" s="17">
+        <v>0.57899999999999996</v>
+      </c>
+      <c r="H16" s="16">
+        <v>89.5</v>
+      </c>
+      <c r="I16" s="17">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="B17" s="16">
+        <v>646240</v>
+      </c>
+      <c r="C17" s="16">
+        <v>19.2</v>
+      </c>
+      <c r="D17" s="16">
+        <v>0.19</v>
+      </c>
+      <c r="E17" s="16">
+        <v>71.8</v>
+      </c>
+      <c r="F17" s="16">
+        <v>14.3</v>
+      </c>
+      <c r="G17" s="17">
+        <v>0.316</v>
+      </c>
+      <c r="H17" s="16">
+        <v>92.2</v>
+      </c>
+      <c r="I17" s="17">
+        <v>0.11700000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="B18" s="16">
+        <v>695578</v>
+      </c>
+      <c r="C18" s="16">
+        <v>29.7</v>
+      </c>
+      <c r="D18" s="16">
+        <v>0.25</v>
+      </c>
+      <c r="E18" s="16">
+        <v>76.8</v>
+      </c>
+      <c r="F18" s="16">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="G18" s="17">
+        <v>0.64300000000000002</v>
+      </c>
+      <c r="H18" s="16">
+        <v>95</v>
+      </c>
+      <c r="I18" s="17">
+        <v>0.22700000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="16" t="s">
+        <v>292</v>
+      </c>
+      <c r="B19" s="16">
+        <v>641343</v>
+      </c>
+      <c r="C19" s="16">
+        <v>15.2</v>
+      </c>
+      <c r="D19" s="16">
+        <v>0.21</v>
+      </c>
+      <c r="E19" s="16">
+        <v>76.8</v>
+      </c>
+      <c r="F19" s="16">
+        <v>11.1</v>
+      </c>
+      <c r="G19" s="17">
+        <v>0.27800000000000002</v>
+      </c>
+      <c r="H19" s="16">
+        <v>92.5</v>
+      </c>
+      <c r="I19" s="17">
+        <v>0.14099999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="B20" s="16">
+        <v>808959</v>
+      </c>
+      <c r="C20" s="16">
+        <v>17.5</v>
+      </c>
+      <c r="D20" s="16">
+        <v>0.31</v>
+      </c>
+      <c r="E20" s="16">
+        <v>75.2</v>
+      </c>
+      <c r="F20" s="16">
+        <v>14</v>
+      </c>
+      <c r="G20" s="17">
+        <v>0.65</v>
+      </c>
+      <c r="H20" s="16">
+        <v>94.1</v>
+      </c>
+      <c r="I20" s="17">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="B21" s="16">
+        <v>691718</v>
+      </c>
+      <c r="C21" s="16">
+        <v>19.8</v>
+      </c>
+      <c r="D21" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E21" s="16">
+        <v>74.8</v>
+      </c>
+      <c r="F21" s="16">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="G21" s="17">
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="H21" s="16">
+        <v>90.2</v>
+      </c>
+      <c r="I21" s="17">
+        <v>0.107</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="16">
+        <v>592518</v>
+      </c>
+      <c r="C22" s="16">
+        <v>17</v>
+      </c>
+      <c r="D22" s="16">
+        <v>0.19</v>
+      </c>
+      <c r="E22" s="16">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="F22" s="16">
+        <v>12.9</v>
+      </c>
+      <c r="G22" s="17">
+        <v>0.158</v>
+      </c>
+      <c r="H22" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I22" s="17">
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="B23" s="16">
+        <v>683002</v>
+      </c>
+      <c r="C23" s="16">
+        <v>15.6</v>
+      </c>
+      <c r="D23" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="E23" s="16">
+        <v>74.400000000000006</v>
+      </c>
+      <c r="F23" s="16">
+        <v>11.9</v>
+      </c>
+      <c r="G23" s="17">
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="H23" s="16">
+        <v>89.7</v>
+      </c>
+      <c r="I23" s="17">
+        <v>7.2999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="16">
+        <v>677594</v>
+      </c>
+      <c r="C24" s="16">
+        <v>15.7</v>
+      </c>
+      <c r="D24" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="E24" s="16">
+        <v>76.5</v>
+      </c>
+      <c r="F24" s="16">
+        <v>12.5</v>
+      </c>
+      <c r="G24" s="17">
+        <v>0.57099999999999995</v>
+      </c>
+      <c r="H24" s="16">
+        <v>90.2</v>
+      </c>
+      <c r="I24" s="17">
+        <v>9.0999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="16">
+        <v>672960</v>
+      </c>
+      <c r="C25" s="16">
+        <v>20.2</v>
+      </c>
+      <c r="D25" s="16">
+        <v>0.23</v>
+      </c>
+      <c r="E25" s="16">
+        <v>73.2</v>
+      </c>
+      <c r="F25" s="16">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="G25" s="17">
+        <v>0.36399999999999999</v>
+      </c>
+      <c r="H25" s="16">
+        <v>91.5</v>
+      </c>
+      <c r="I25" s="17">
+        <v>0.14799999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="B26" s="16">
+        <v>694212</v>
+      </c>
+      <c r="C26" s="16">
+        <v>13</v>
+      </c>
+      <c r="D26" s="16">
+        <v>0.21</v>
+      </c>
+      <c r="E26" s="16">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="F26" s="16">
+        <v>11.3</v>
+      </c>
+      <c r="G26" s="17">
+        <v>0.313</v>
+      </c>
+      <c r="H26" s="16">
+        <v>91.5</v>
+      </c>
+      <c r="I26" s="17">
+        <v>0.13100000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="16">
+        <v>545361</v>
+      </c>
+      <c r="C27" s="16">
+        <v>20.9</v>
+      </c>
+      <c r="D27" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E27" s="16">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="F27" s="16">
+        <v>18.2</v>
+      </c>
+      <c r="G27" s="17">
+        <v>0.61099999999999999</v>
+      </c>
+      <c r="H27" s="16">
+        <v>90.7</v>
+      </c>
+      <c r="I27" s="17">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="B28" s="16">
+        <v>665833</v>
+      </c>
+      <c r="C28" s="16">
+        <v>13.8</v>
+      </c>
+      <c r="D28" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E28" s="16">
+        <v>78.5</v>
+      </c>
+      <c r="F28" s="16">
+        <v>7.6</v>
+      </c>
+      <c r="G28" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="H28" s="16">
+        <v>96</v>
+      </c>
+      <c r="I28" s="17">
+        <v>0.16700000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="B29" s="16">
+        <v>547180</v>
+      </c>
+      <c r="C29" s="16">
+        <v>17.3</v>
+      </c>
+      <c r="D29" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E29" s="16">
+        <v>74.3</v>
+      </c>
+      <c r="F29" s="16">
+        <v>11.6</v>
+      </c>
+      <c r="G29" s="17">
+        <v>0.35</v>
+      </c>
+      <c r="H29" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I29" s="17">
+        <v>0.113</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="16">
+        <v>592450</v>
+      </c>
+      <c r="C30" s="16">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="D30" s="16">
+        <v>0.26</v>
+      </c>
+      <c r="E30" s="16">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="F30" s="16">
+        <v>14.6</v>
+      </c>
+      <c r="G30" s="17">
+        <v>0.64700000000000002</v>
+      </c>
+      <c r="H30" s="16">
+        <v>94.1</v>
+      </c>
+      <c r="I30" s="17">
+        <v>0.217</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="B31" s="16">
+        <v>682985</v>
+      </c>
+      <c r="C31" s="16">
+        <v>12.3</v>
+      </c>
+      <c r="D31" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E31" s="16">
+        <v>75.7</v>
+      </c>
+      <c r="F31" s="16">
+        <v>18.2</v>
+      </c>
+      <c r="G31" s="17">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="H31" s="16">
+        <v>91.4</v>
+      </c>
+      <c r="I31" s="17">
+        <v>0.13800000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" s="16" t="s">
+        <v>460</v>
+      </c>
+      <c r="B32" s="16">
+        <v>606466</v>
+      </c>
+      <c r="C32" s="16">
+        <v>18.3</v>
+      </c>
+      <c r="D32" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E32" s="16">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="F32" s="16">
+        <v>12.4</v>
+      </c>
+      <c r="G32" s="17">
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="H32" s="16">
+        <v>91</v>
+      </c>
+      <c r="I32" s="17">
+        <v>0.109</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="16" t="s">
+        <v>461</v>
+      </c>
+      <c r="B33" s="16">
+        <v>664023</v>
+      </c>
+      <c r="C33" s="16">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="D33" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E33" s="16">
+        <v>72.2</v>
+      </c>
+      <c r="F33" s="16">
+        <v>15.8</v>
+      </c>
+      <c r="G33" s="17">
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="H33" s="16">
+        <v>89.6</v>
+      </c>
+      <c r="I33" s="17">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="16">
+        <v>681624</v>
+      </c>
+      <c r="C34" s="16">
+        <v>14.5</v>
+      </c>
+      <c r="D34" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E34" s="16">
+        <v>73</v>
+      </c>
+      <c r="F34" s="16">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="G34" s="17">
+        <v>0.47099999999999997</v>
+      </c>
+      <c r="H34" s="16">
+        <v>89.1</v>
+      </c>
+      <c r="I34" s="17">
+        <v>8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="B35" s="16">
+        <v>660271</v>
+      </c>
+      <c r="C35" s="16">
+        <v>19.7</v>
+      </c>
+      <c r="D35" s="16">
+        <v>0.22</v>
+      </c>
+      <c r="E35" s="16">
+        <v>74.7</v>
+      </c>
+      <c r="F35" s="16">
+        <v>12.8</v>
+      </c>
+      <c r="G35" s="17">
+        <v>0.318</v>
+      </c>
+      <c r="H35" s="16">
+        <v>93.6</v>
+      </c>
+      <c r="I35" s="17">
+        <v>0.17100000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="B36" s="16">
+        <v>664040</v>
+      </c>
+      <c r="C36" s="16">
+        <v>21.7</v>
+      </c>
+      <c r="D36" s="16">
+        <v>0.21</v>
+      </c>
+      <c r="E36" s="16">
+        <v>73.7</v>
+      </c>
+      <c r="F36" s="16">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="G36" s="17">
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="H36" s="16">
+        <v>90.9</v>
+      </c>
+      <c r="I36" s="17">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="B37" s="16">
+        <v>668709</v>
+      </c>
+      <c r="C37" s="16">
+        <v>13.4</v>
+      </c>
+      <c r="D37" s="16">
+        <v>0.23</v>
+      </c>
+      <c r="E37" s="16">
+        <v>73.8</v>
+      </c>
+      <c r="F37" s="16">
+        <v>21.2</v>
+      </c>
+      <c r="G37" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="H37" s="16">
+        <v>89</v>
+      </c>
+      <c r="I37" s="17">
+        <v>0.10299999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A38" s="16" t="s">
+        <v>462</v>
+      </c>
+      <c r="B38" s="16">
+        <v>682829</v>
+      </c>
+      <c r="C38" s="16">
+        <v>13.4</v>
+      </c>
+      <c r="D38" s="16">
+        <v>0.18</v>
+      </c>
+      <c r="E38" s="16">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="F38" s="16">
+        <v>11.1</v>
+      </c>
+      <c r="G38" s="17">
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="H38" s="16">
+        <v>94.4</v>
+      </c>
+      <c r="I38" s="17">
+        <v>0.153</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="B39" s="16">
+        <v>686527</v>
+      </c>
+      <c r="C39" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="D39" s="16">
+        <v>0.24</v>
+      </c>
+      <c r="E39" s="16">
+        <v>74.8</v>
+      </c>
+      <c r="F39" s="16">
+        <v>9.6</v>
+      </c>
+      <c r="G39" s="17">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="H39" s="16">
+        <v>92.8</v>
+      </c>
+      <c r="I39" s="17">
+        <v>0.153</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" s="16">
+        <v>701398</v>
+      </c>
+      <c r="C40" s="16">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="D40" s="16">
+        <v>0.18</v>
+      </c>
+      <c r="E40" s="16">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="F40" s="16">
+        <v>13.8</v>
+      </c>
+      <c r="G40" s="17">
+        <v>0.158</v>
+      </c>
+      <c r="H40" s="16">
+        <v>90.6</v>
+      </c>
+      <c r="I40" s="17">
+        <v>0.14899999999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B41" s="16">
+        <v>678554</v>
+      </c>
+      <c r="C41" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="D41" s="16">
+        <v>0.23</v>
+      </c>
+      <c r="E41" s="16">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="F41" s="16">
+        <v>15.8</v>
+      </c>
+      <c r="G41" s="17">
+        <v>0.52900000000000003</v>
+      </c>
+      <c r="H41" s="16">
+        <v>87.9</v>
+      </c>
+      <c r="I41" s="17">
+        <v>0.11899999999999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" s="16" t="s">
+        <v>309</v>
+      </c>
+      <c r="B42" s="16">
+        <v>691016</v>
+      </c>
+      <c r="C42" s="16">
+        <v>9.1</v>
+      </c>
+      <c r="D42" s="16">
+        <v>0.16</v>
+      </c>
+      <c r="E42" s="16">
+        <v>74.5</v>
+      </c>
+      <c r="F42" s="16">
+        <v>12</v>
+      </c>
+      <c r="G42" s="17">
+        <v>0.214</v>
+      </c>
+      <c r="H42" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I42" s="17">
+        <v>0.10100000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="16">
+        <v>575929</v>
+      </c>
+      <c r="C43" s="16">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="D43" s="16">
+        <v>0.22</v>
+      </c>
+      <c r="E43" s="16">
+        <v>77</v>
+      </c>
+      <c r="F43" s="16">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="G43" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="H43" s="16">
+        <v>90.6</v>
+      </c>
+      <c r="I43" s="17">
+        <v>0.14299999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="B44" s="16">
+        <v>665862</v>
+      </c>
+      <c r="C44" s="16">
+        <v>13.1</v>
+      </c>
+      <c r="D44" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E44" s="16">
+        <v>73.099999999999994</v>
+      </c>
+      <c r="F44" s="16">
+        <v>16.2</v>
+      </c>
+      <c r="G44" s="17">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="H44" s="16">
+        <v>90.7</v>
+      </c>
+      <c r="I44" s="17">
+        <v>8.7999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="B45" s="16">
+        <v>686948</v>
+      </c>
+      <c r="C45" s="16">
+        <v>12.6</v>
+      </c>
+      <c r="D45" s="16">
+        <v>0.19</v>
+      </c>
+      <c r="E45" s="16">
+        <v>75</v>
+      </c>
+      <c r="F45" s="16">
+        <v>11.4</v>
+      </c>
+      <c r="G45" s="17">
+        <v>0.2</v>
+      </c>
+      <c r="H45" s="16">
+        <v>91.4</v>
+      </c>
+      <c r="I45" s="17">
+        <v>0.153</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="B46" s="16">
+        <v>621566</v>
+      </c>
+      <c r="C46" s="16">
+        <v>25.7</v>
+      </c>
+      <c r="D46" s="16">
+        <v>0.24</v>
+      </c>
+      <c r="E46" s="16">
+        <v>75</v>
+      </c>
+      <c r="F46" s="16">
+        <v>17.7</v>
+      </c>
+      <c r="G46" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="H46" s="16">
+        <v>92.9</v>
+      </c>
+      <c r="I46" s="17">
+        <v>0.13900000000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" s="16" t="s">
+        <v>294</v>
+      </c>
+      <c r="B47" s="16">
+        <v>671739</v>
+      </c>
+      <c r="C47" s="16">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="D47" s="16">
+        <v>0.18</v>
+      </c>
+      <c r="E47" s="16">
+        <v>74.8</v>
+      </c>
+      <c r="F47" s="16">
+        <v>10.4</v>
+      </c>
+      <c r="G47" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="H47" s="16">
+        <v>91.7</v>
+      </c>
+      <c r="I47" s="17">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B48" s="16">
+        <v>678246</v>
+      </c>
+      <c r="C48" s="16">
+        <v>22.6</v>
+      </c>
+      <c r="D48" s="16">
+        <v>0.21</v>
+      </c>
+      <c r="E48" s="16">
+        <v>74.099999999999994</v>
+      </c>
+      <c r="F48" s="16">
+        <v>19.7</v>
+      </c>
+      <c r="G48" s="17">
+        <v>0.57099999999999995</v>
+      </c>
+      <c r="H48" s="16">
+        <v>90.6</v>
+      </c>
+      <c r="I48" s="17">
+        <v>0.154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="B49" s="16">
+        <v>682928</v>
+      </c>
+      <c r="C49" s="16">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="D49" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E49" s="16">
+        <v>72.8</v>
+      </c>
+      <c r="F49" s="16">
+        <v>18.7</v>
+      </c>
+      <c r="G49" s="17">
+        <v>0.3</v>
+      </c>
+      <c r="H49" s="16">
+        <v>89.9</v>
+      </c>
+      <c r="I49" s="17">
+        <v>9.8000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B50" s="16">
+        <v>694192</v>
+      </c>
+      <c r="C50" s="16">
+        <v>9.9</v>
+      </c>
+      <c r="D50" s="16">
+        <v>0.18</v>
+      </c>
+      <c r="E50" s="16">
+        <v>74.8</v>
+      </c>
+      <c r="F50" s="16">
+        <v>13.5</v>
+      </c>
+      <c r="G50" s="17">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="H50" s="16">
+        <v>92.2</v>
+      </c>
+      <c r="I50" s="17">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51" s="16" t="s">
+        <v>325</v>
+      </c>
+      <c r="B51" s="16">
+        <v>641355</v>
+      </c>
+      <c r="C51" s="16">
+        <v>9.1</v>
+      </c>
+      <c r="D51" s="16">
+        <v>0.11</v>
+      </c>
+      <c r="E51" s="16">
+        <v>69.5</v>
+      </c>
+      <c r="F51" s="16">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="G51" s="17">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="H51" s="16">
+        <v>88.9</v>
+      </c>
+      <c r="I51" s="17">
+        <v>6.6000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A52" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="B52" s="16">
+        <v>670042</v>
+      </c>
+      <c r="C52" s="16">
+        <v>12.7</v>
+      </c>
+      <c r="D52" s="16">
+        <v>0.22</v>
+      </c>
+      <c r="E52" s="16">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="F52" s="16">
+        <v>15.5</v>
+      </c>
+      <c r="G52" s="17">
+        <v>0.35699999999999998</v>
+      </c>
+      <c r="H52" s="16">
+        <v>90.6</v>
+      </c>
+      <c r="I52" s="17">
+        <v>0.161</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A53" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" s="16">
+        <v>571448</v>
+      </c>
+      <c r="C53" s="16">
+        <v>10.4</v>
+      </c>
+      <c r="D53" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E53" s="16">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="F53" s="16">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="G53" s="17">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="H53" s="16">
+        <v>85.2</v>
+      </c>
+      <c r="I53" s="17">
+        <v>7.0999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A54" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B54" s="16">
+        <v>521692</v>
+      </c>
+      <c r="C54" s="16">
+        <v>11.9</v>
+      </c>
+      <c r="D54" s="16">
+        <v>0.12</v>
+      </c>
+      <c r="E54" s="16">
+        <v>71.8</v>
+      </c>
+      <c r="F54" s="16">
+        <v>16.5</v>
+      </c>
+      <c r="G54" s="17">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="H54" s="16">
+        <v>89.3</v>
+      </c>
+      <c r="I54" s="17">
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A55" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="B55" s="16">
+        <v>592626</v>
+      </c>
+      <c r="C55" s="16">
+        <v>12.1</v>
+      </c>
+      <c r="D55" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E55" s="16">
+        <v>72</v>
+      </c>
+      <c r="F55" s="16">
+        <v>14.6</v>
+      </c>
+      <c r="G55" s="17">
+        <v>0.4</v>
+      </c>
+      <c r="H55" s="16">
+        <v>91.9</v>
+      </c>
+      <c r="I55" s="17">
+        <v>0.112</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A56" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="B56" s="16">
+        <v>666160</v>
+      </c>
+      <c r="C56" s="16">
+        <v>12.7</v>
+      </c>
+      <c r="D56" s="16">
+        <v>0.26</v>
+      </c>
+      <c r="E56" s="16">
+        <v>74.400000000000006</v>
+      </c>
+      <c r="F56" s="16">
+        <v>22.6</v>
+      </c>
+      <c r="G56" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="H56" s="16">
+        <v>89.6</v>
+      </c>
+      <c r="I56" s="17">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A57" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="B57" s="16">
+        <v>571970</v>
+      </c>
+      <c r="C57" s="16">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="D57" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E57" s="16">
+        <v>71.5</v>
+      </c>
+      <c r="F57" s="16">
+        <v>14.8</v>
+      </c>
+      <c r="G57" s="17">
+        <v>0.47099999999999997</v>
+      </c>
+      <c r="H57" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I57" s="17">
+        <v>0.13600000000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A58" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B58" s="16">
+        <v>693307</v>
+      </c>
+      <c r="C58" s="16">
+        <v>17.5</v>
+      </c>
+      <c r="D58" s="16">
+        <v>0.21</v>
+      </c>
+      <c r="E58" s="16">
+        <v>72</v>
+      </c>
+      <c r="F58" s="16">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="G58" s="17">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="H58" s="16">
+        <v>89.7</v>
+      </c>
+      <c r="I58" s="17">
+        <v>0.11600000000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A59" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B59" s="16">
+        <v>670623</v>
+      </c>
+      <c r="C59" s="16">
+        <v>10.8</v>
+      </c>
+      <c r="D59" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E59" s="16">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="F59" s="16">
+        <v>24</v>
+      </c>
+      <c r="G59" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="H59" s="16">
+        <v>86.7</v>
+      </c>
+      <c r="I59" s="17">
+        <v>5.8999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A60" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="B60" s="16">
+        <v>695600</v>
+      </c>
+      <c r="C60" s="16">
+        <v>12.2</v>
+      </c>
+      <c r="D60" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="E60" s="16">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="F60" s="16">
+        <v>20.2</v>
+      </c>
+      <c r="G60" s="17">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="H60" s="16">
+        <v>90.8</v>
+      </c>
+      <c r="I60" s="17">
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A61" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="B61" s="16">
+        <v>656811</v>
+      </c>
+      <c r="C61" s="16">
+        <v>15.6</v>
+      </c>
+      <c r="D61" s="16">
+        <v>0.19</v>
+      </c>
+      <c r="E61" s="16">
+        <v>70.8</v>
+      </c>
+      <c r="F61" s="16">
+        <v>13.7</v>
+      </c>
+      <c r="G61" s="17">
+        <v>6.3E-2</v>
+      </c>
+      <c r="H61" s="16">
+        <v>89.7</v>
+      </c>
+      <c r="I61" s="17">
+        <v>8.1000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A62" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B62" s="16">
+        <v>621020</v>
+      </c>
+      <c r="C62" s="16">
+        <v>13</v>
+      </c>
+      <c r="D62" s="16">
+        <v>0.18</v>
+      </c>
+      <c r="E62" s="16">
+        <v>71.5</v>
+      </c>
+      <c r="F62" s="16">
+        <v>16.8</v>
+      </c>
+      <c r="G62" s="17">
+        <v>0.438</v>
+      </c>
+      <c r="H62" s="16">
+        <v>89.9</v>
+      </c>
+      <c r="I62" s="17">
+        <v>7.6999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A63" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B63" s="16">
+        <v>669477</v>
+      </c>
+      <c r="C63" s="16">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="D63" s="16">
+        <v>0.21</v>
+      </c>
+      <c r="E63" s="16">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="F63" s="16">
+        <v>21.5</v>
+      </c>
+      <c r="G63" s="17">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="H63" s="16">
+        <v>90</v>
+      </c>
+      <c r="I63" s="17">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A64" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B64" s="16">
+        <v>621493</v>
+      </c>
+      <c r="C64" s="16">
+        <v>6</v>
+      </c>
+      <c r="D64" s="16">
+        <v>0.05</v>
+      </c>
+      <c r="E64" s="16">
+        <v>68.2</v>
+      </c>
+      <c r="F64" s="16">
+        <v>14.6</v>
+      </c>
+      <c r="G64" s="17">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="H64" s="16">
+        <v>89.4</v>
+      </c>
+      <c r="I64" s="17">
+        <v>5.6000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="16" t="s">
+        <v>482</v>
+      </c>
+      <c r="B65" s="16">
+        <v>596019</v>
+      </c>
+      <c r="C65" s="16">
+        <v>5.7</v>
+      </c>
+      <c r="D65" s="16">
+        <v>0.12</v>
+      </c>
+      <c r="E65" s="16">
+        <v>72.599999999999994</v>
+      </c>
+      <c r="F65" s="16">
+        <v>14.8</v>
+      </c>
+      <c r="G65" s="17">
+        <v>0.6</v>
+      </c>
+      <c r="H65" s="16">
+        <v>92</v>
+      </c>
+      <c r="I65" s="17">
+        <v>8.6999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B66" s="16">
+        <v>673548</v>
+      </c>
+      <c r="C66" s="16">
+        <v>15.4</v>
+      </c>
+      <c r="D66" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E66" s="16">
+        <v>73.3</v>
+      </c>
+      <c r="F66" s="16">
+        <v>18.3</v>
+      </c>
+      <c r="G66" s="17">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="H66" s="16">
+        <v>89</v>
+      </c>
+      <c r="I66" s="17">
+        <v>9.1999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="B67" s="16">
+        <v>695506</v>
+      </c>
+      <c r="C67" s="16">
+        <v>15.6</v>
+      </c>
+      <c r="D67" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E67" s="16">
+        <v>77.3</v>
+      </c>
+      <c r="F67" s="16">
+        <v>7.3</v>
+      </c>
+      <c r="G67" s="17">
+        <v>0.73299999999999998</v>
+      </c>
+      <c r="H67" s="16">
+        <v>93</v>
+      </c>
+      <c r="I67" s="17">
+        <v>0.14699999999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A68" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B68" s="16">
+        <v>605141</v>
+      </c>
+      <c r="C68" s="16">
+        <v>8.1</v>
+      </c>
+      <c r="D68" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E68" s="16">
+        <v>69.5</v>
+      </c>
+      <c r="F68" s="16">
+        <v>19</v>
+      </c>
+      <c r="G68" s="17">
+        <v>9.0999999999999998E-2</v>
+      </c>
+      <c r="H68" s="16">
+        <v>90.5</v>
+      </c>
+      <c r="I68" s="17">
+        <v>8.1000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A69" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="B69" s="16">
+        <v>701538</v>
+      </c>
+      <c r="C69" s="16">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="D69" s="16">
+        <v>0.1</v>
+      </c>
+      <c r="E69" s="16">
+        <v>73.400000000000006</v>
+      </c>
+      <c r="F69" s="16">
+        <v>12.9</v>
+      </c>
+      <c r="G69" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="H69" s="16">
+        <v>89.4</v>
+      </c>
+      <c r="I69" s="17">
+        <v>9.0999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A70" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B70" s="16">
+        <v>661388</v>
+      </c>
+      <c r="C70" s="16">
+        <v>7.9</v>
+      </c>
+      <c r="D70" s="16">
+        <v>0.09</v>
+      </c>
+      <c r="E70" s="16">
+        <v>73.2</v>
+      </c>
+      <c r="F70" s="16">
+        <v>11.8</v>
+      </c>
+      <c r="G70" s="17">
+        <v>0.55600000000000005</v>
+      </c>
+      <c r="H70" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I70" s="17">
+        <v>7.0999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A71" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="B71" s="16">
+        <v>669016</v>
+      </c>
+      <c r="C71" s="16">
+        <v>11.1</v>
+      </c>
+      <c r="D71" s="16">
+        <v>0.17</v>
+      </c>
+      <c r="E71" s="16">
+        <v>71.5</v>
+      </c>
+      <c r="F71" s="16">
+        <v>13.2</v>
+      </c>
+      <c r="G71" s="17">
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="H71" s="16">
+        <v>89.8</v>
+      </c>
+      <c r="I71" s="17">
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A72" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B72" s="16">
+        <v>553993</v>
+      </c>
+      <c r="C72" s="16">
+        <v>8.6</v>
+      </c>
+      <c r="D72" s="16">
+        <v>0.16</v>
+      </c>
+      <c r="E72" s="16">
+        <v>71.5</v>
+      </c>
+      <c r="F72" s="16">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="G72" s="17">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="H72" s="16">
+        <v>87.9</v>
+      </c>
+      <c r="I72" s="17">
+        <v>9.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A73" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B73" s="16">
+        <v>514888</v>
+      </c>
+      <c r="C73" s="16">
+        <v>9.4</v>
+      </c>
+      <c r="D73" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E73" s="16">
+        <v>68.7</v>
+      </c>
+      <c r="F73" s="16">
+        <v>9.5</v>
+      </c>
+      <c r="G73" s="17">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="H73" s="16">
+        <v>85.8</v>
+      </c>
+      <c r="I73" s="17">
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A74" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B74" s="16">
+        <v>642715</v>
+      </c>
+      <c r="C74" s="16">
+        <v>14.6</v>
+      </c>
+      <c r="D74" s="16">
+        <v>0.16</v>
+      </c>
+      <c r="E74" s="16">
+        <v>72.3</v>
+      </c>
+      <c r="F74" s="16">
+        <v>22.2</v>
+      </c>
+      <c r="G74" s="17">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="H74" s="16">
+        <v>88.4</v>
+      </c>
+      <c r="I74" s="17">
+        <v>8.7999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A75" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B75" s="16">
+        <v>666182</v>
+      </c>
+      <c r="C75" s="16">
+        <v>10.1</v>
+      </c>
+      <c r="D75" s="16">
+        <v>0.1</v>
+      </c>
+      <c r="E75" s="16">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="F75" s="16">
+        <v>8.5</v>
+      </c>
+      <c r="G75" s="17">
+        <v>0.3</v>
+      </c>
+      <c r="H75" s="16">
+        <v>90.3</v>
+      </c>
+      <c r="I75" s="17">
+        <v>7.0999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A76" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B76" s="16">
+        <v>624585</v>
+      </c>
+      <c r="C76" s="16">
+        <v>11.2</v>
+      </c>
+      <c r="D76" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E76" s="16">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="F76" s="16">
+        <v>14.5</v>
+      </c>
+      <c r="G76" s="17">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="H76" s="16">
+        <v>88.2</v>
+      </c>
+      <c r="I76" s="17">
+        <v>0.11700000000000001</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A77" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B77" s="16">
+        <v>607208</v>
+      </c>
+      <c r="C77" s="16">
+        <v>8.4</v>
+      </c>
+      <c r="D77" s="16">
+        <v>0.1</v>
+      </c>
+      <c r="E77" s="16">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="F77" s="16">
+        <v>10.1</v>
+      </c>
+      <c r="G77" s="17">
+        <v>0.4</v>
+      </c>
+      <c r="H77" s="16">
+        <v>88.6</v>
+      </c>
+      <c r="I77" s="17">
+        <v>6.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A78" s="16" t="s">
+        <v>465</v>
+      </c>
+      <c r="B78" s="16">
+        <v>686797</v>
+      </c>
+      <c r="C78" s="16">
+        <v>10.6</v>
+      </c>
+      <c r="D78" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="E78" s="16">
+        <v>70.2</v>
+      </c>
+      <c r="F78" s="16">
+        <v>15</v>
+      </c>
+      <c r="G78" s="17">
+        <v>0.28599999999999998</v>
+      </c>
+      <c r="H78" s="16">
+        <v>88</v>
+      </c>
+      <c r="I78" s="17">
+        <v>3.9E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A79" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="B79" s="16">
+        <v>802139</v>
+      </c>
+      <c r="C79" s="16">
+        <v>11.2</v>
+      </c>
+      <c r="D79" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E79" s="16">
+        <v>72.400000000000006</v>
+      </c>
+      <c r="F79" s="16">
+        <v>13.7</v>
+      </c>
+      <c r="G79" s="17">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="H79" s="16">
+        <v>90</v>
+      </c>
+      <c r="I79" s="17">
+        <v>7.2999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A80" s="16" t="s">
+        <v>466</v>
+      </c>
+      <c r="B80" s="16">
+        <v>605137</v>
+      </c>
+      <c r="C80" s="16">
+        <v>14.9</v>
+      </c>
+      <c r="D80" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E80" s="16">
+        <v>72.099999999999994</v>
+      </c>
+      <c r="F80" s="16">
+        <v>14.1</v>
+      </c>
+      <c r="G80" s="17">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="H80" s="16">
+        <v>89.9</v>
+      </c>
+      <c r="I80" s="17">
+        <v>0.106</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A81" s="16" t="s">
+        <v>464</v>
+      </c>
+      <c r="B81" s="16">
+        <v>645277</v>
+      </c>
+      <c r="C81" s="16">
+        <v>13</v>
+      </c>
+      <c r="D81" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E81" s="16">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="F81" s="16">
+        <v>17.5</v>
+      </c>
+      <c r="G81" s="17">
+        <v>0.42899999999999999</v>
+      </c>
+      <c r="H81" s="16">
+        <v>87.2</v>
+      </c>
+      <c r="I81" s="17">
+        <v>4.1000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A82" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="B82" s="16">
+        <v>668930</v>
+      </c>
+      <c r="C82" s="16">
+        <v>10.6</v>
+      </c>
+      <c r="D82" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E82" s="16">
+        <v>70</v>
+      </c>
+      <c r="F82" s="16">
+        <v>7.9</v>
+      </c>
+      <c r="G82" s="17">
+        <v>0.214</v>
+      </c>
+      <c r="H82" s="16">
+        <v>90.9</v>
+      </c>
+      <c r="I82" s="17">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A83" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B83" s="16">
+        <v>650490</v>
+      </c>
+      <c r="C83" s="16">
+        <v>13.9</v>
+      </c>
+      <c r="D83" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E83" s="16">
+        <v>73.8</v>
+      </c>
+      <c r="F83" s="16">
+        <v>6</v>
+      </c>
+      <c r="G83" s="17">
+        <v>0.38500000000000001</v>
+      </c>
+      <c r="H83" s="16">
+        <v>91.1</v>
+      </c>
+      <c r="I83" s="17">
+        <v>7.0999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A84" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B84" s="16">
+        <v>682998</v>
+      </c>
+      <c r="C84" s="16">
+        <v>15</v>
+      </c>
+      <c r="D84" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E84" s="16">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="F84" s="16">
+        <v>13.2</v>
+      </c>
+      <c r="G84" s="17">
+        <v>0.38500000000000001</v>
+      </c>
+      <c r="H84" s="16">
+        <v>91.3</v>
+      </c>
+      <c r="I84" s="17">
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A85" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B85" s="16">
+        <v>666176</v>
+      </c>
+      <c r="C85" s="16">
+        <v>14.8</v>
+      </c>
+      <c r="D85" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E85" s="16">
+        <v>77.3</v>
+      </c>
+      <c r="F85" s="16">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="G85" s="17">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="H85" s="16">
+        <v>89.7</v>
+      </c>
+      <c r="I85" s="17">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A86" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B86" s="16">
+        <v>677951</v>
+      </c>
+      <c r="C86" s="16">
+        <v>11</v>
+      </c>
+      <c r="D86" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E86" s="16">
+        <v>73.7</v>
+      </c>
+      <c r="F86" s="16">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="G86" s="17">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="H86" s="16">
+        <v>93.2</v>
+      </c>
+      <c r="I86" s="17">
+        <v>0.121</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A87" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="B87" s="16">
+        <v>702616</v>
+      </c>
+      <c r="C87" s="16">
+        <v>3.7</v>
+      </c>
+      <c r="D87" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E87" s="16">
+        <v>70.5</v>
+      </c>
+      <c r="F87" s="16">
+        <v>12.7</v>
+      </c>
+      <c r="G87" s="17">
+        <v>0.2</v>
+      </c>
+      <c r="H87" s="16">
+        <v>87.3</v>
+      </c>
+      <c r="I87" s="17">
+        <v>0.107</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A88" s="16" t="s">
+        <v>328</v>
+      </c>
+      <c r="B88" s="16">
+        <v>702284</v>
+      </c>
+      <c r="C88" s="16">
+        <v>11</v>
+      </c>
+      <c r="D88" s="16">
+        <v>0.11</v>
+      </c>
+      <c r="E88" s="16">
+        <v>71.7</v>
+      </c>
+      <c r="F88" s="16">
+        <v>14.7</v>
+      </c>
+      <c r="G88" s="17">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="H88" s="16">
+        <v>88.6</v>
+      </c>
+      <c r="I88" s="17">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A89" s="16" t="s">
+        <v>470</v>
+      </c>
+      <c r="B89" s="16">
+        <v>641680</v>
+      </c>
+      <c r="C89" s="16">
+        <v>7.7</v>
+      </c>
+      <c r="D89" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="E89" s="16">
+        <v>70.2</v>
+      </c>
+      <c r="F89" s="16">
+        <v>11.6</v>
+      </c>
+      <c r="G89" s="17">
+        <v>0.222</v>
+      </c>
+      <c r="H89" s="16">
+        <v>87.1</v>
+      </c>
+      <c r="I89" s="17">
+        <v>6.9000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A90" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B90" s="16">
+        <v>660670</v>
+      </c>
+      <c r="C90" s="16">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="D90" s="16">
+        <v>0.12</v>
+      </c>
+      <c r="E90" s="16">
+        <v>76</v>
+      </c>
+      <c r="F90" s="16">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="G90" s="17">
+        <v>0.71399999999999997</v>
+      </c>
+      <c r="H90" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I90" s="17">
+        <v>0.13100000000000001</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A91" s="16" t="s">
+        <v>326</v>
+      </c>
+      <c r="B91" s="16">
+        <v>677800</v>
+      </c>
+      <c r="C91" s="16">
+        <v>13.5</v>
+      </c>
+      <c r="D91" s="16">
+        <v>0.11</v>
+      </c>
+      <c r="E91" s="16">
+        <v>73.8</v>
+      </c>
+      <c r="F91" s="16">
+        <v>18.3</v>
+      </c>
+      <c r="G91" s="17">
+        <v>0.36399999999999999</v>
+      </c>
+      <c r="H91" s="16">
+        <v>90.1</v>
+      </c>
+      <c r="I91" s="17">
+        <v>0.123</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A92" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B92" s="16">
+        <v>676391</v>
+      </c>
+      <c r="C92" s="16">
+        <v>7.5</v>
+      </c>
+      <c r="D92" s="16">
+        <v>0.09</v>
+      </c>
+      <c r="E92" s="16">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="F92" s="16">
+        <v>15.9</v>
+      </c>
+      <c r="G92" s="17">
+        <v>0.125</v>
+      </c>
+      <c r="H92" s="16">
+        <v>85.2</v>
+      </c>
+      <c r="I92" s="17">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A93" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="B93" s="16">
+        <v>683953</v>
+      </c>
+      <c r="C93" s="16">
+        <v>7.4</v>
+      </c>
+      <c r="D93" s="16">
+        <v>0.1</v>
+      </c>
+      <c r="E93" s="16">
+        <v>69.8</v>
+      </c>
+      <c r="F93" s="16">
+        <v>14.5</v>
+      </c>
+      <c r="G93" s="17">
+        <v>0.28599999999999998</v>
+      </c>
+      <c r="H93" s="16">
+        <v>88.1</v>
+      </c>
+      <c r="I93" s="17">
+        <v>4.2999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A94" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="B94" s="16">
+        <v>689414</v>
+      </c>
+      <c r="C94" s="16">
+        <v>11.6</v>
+      </c>
+      <c r="D94" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="E94" s="16">
+        <v>68.5</v>
+      </c>
+      <c r="F94" s="16">
+        <v>13.5</v>
+      </c>
+      <c r="G94" s="17">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="H94" s="16">
+        <v>85.4</v>
+      </c>
+      <c r="I94" s="17">
+        <v>3.5999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A95" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="B95" s="16">
+        <v>664983</v>
+      </c>
+      <c r="C95" s="16">
+        <v>7.8</v>
+      </c>
+      <c r="D95" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E95" s="16">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="F95" s="16">
+        <v>12.3</v>
+      </c>
+      <c r="G95" s="17">
+        <v>0.4</v>
+      </c>
+      <c r="H95" s="16">
+        <v>85</v>
+      </c>
+      <c r="I95" s="17">
+        <v>6.0999999999999999E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Home ticker + Dataroom, spray-chart fix, recap fixes, new Mickey tiers
</commit_message>
<xml_diff>
--- a/data/dingers_player_data.xlsx
+++ b/data/dingers_player_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshbrodie/Desktop/claude_code/dingers/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4083E013-0051-D84D-A88A-542726E47F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758FA0BD-743E-9C42-B57F-3C4AE3AE9651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="720" yWindow="1040" windowWidth="27240" windowHeight="16180" activeTab="6" xr2:uid="{60B155BA-D1AB-C646-8118-9D9B551D7988}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6595" uniqueCount="2307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6600" uniqueCount="2307">
   <si>
     <t>Rk</t>
   </si>
@@ -91731,7 +91731,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6B2B3E9-7332-1E40-9045-0257B743AEA0}">
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
@@ -94489,6 +94489,151 @@
         <v>6.0999999999999999E-2</v>
       </c>
     </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A96" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="B96" s="16">
+        <v>663757</v>
+      </c>
+      <c r="C96" s="16">
+        <v>9</v>
+      </c>
+      <c r="D96" s="16">
+        <v>0.13</v>
+      </c>
+      <c r="E96" s="16">
+        <v>70.2</v>
+      </c>
+      <c r="F96" s="16">
+        <v>17.3</v>
+      </c>
+      <c r="G96" s="17">
+        <v>0.4</v>
+      </c>
+      <c r="H96" s="16">
+        <v>91.1</v>
+      </c>
+      <c r="I96" s="17">
+        <v>0.109</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A97" s="16" t="s">
+        <v>350</v>
+      </c>
+      <c r="B97" s="16">
+        <v>805811</v>
+      </c>
+      <c r="C97" s="16">
+        <v>8.5</v>
+      </c>
+      <c r="D97" s="16">
+        <v>0.15</v>
+      </c>
+      <c r="E97" s="16">
+        <v>73.7</v>
+      </c>
+      <c r="F97" s="16">
+        <v>13.2</v>
+      </c>
+      <c r="G97" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="H97" s="16">
+        <v>92.3</v>
+      </c>
+      <c r="I97" s="17">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A98" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B98" s="16">
+        <v>671056</v>
+      </c>
+      <c r="C98" s="16">
+        <v>11.7</v>
+      </c>
+      <c r="D98" s="16">
+        <v>0.1</v>
+      </c>
+      <c r="E98" s="16">
+        <v>73.900000000000006</v>
+      </c>
+      <c r="F98" s="16">
+        <v>9.4</v>
+      </c>
+      <c r="G98" s="17">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="H98" s="16">
+        <v>89.2</v>
+      </c>
+      <c r="I98" s="17">
+        <v>5.8000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A99" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="B99" s="16">
+        <v>681297</v>
+      </c>
+      <c r="C99" s="16">
+        <v>7.9</v>
+      </c>
+      <c r="D99" s="16">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E99" s="16">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="F99" s="16">
+        <v>13.2</v>
+      </c>
+      <c r="G99" s="17">
+        <v>0.875</v>
+      </c>
+      <c r="H99" s="16">
+        <v>86.8</v>
+      </c>
+      <c r="I99" s="17">
+        <v>0.113</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A100" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B100" s="16">
+        <v>668904</v>
+      </c>
+      <c r="C100" s="16">
+        <v>11.7</v>
+      </c>
+      <c r="D100" s="16">
+        <v>0.16</v>
+      </c>
+      <c r="E100" s="16">
+        <v>74.5</v>
+      </c>
+      <c r="F100" s="16">
+        <v>19.7</v>
+      </c>
+      <c r="G100" s="17">
+        <v>0.7</v>
+      </c>
+      <c r="H100" s="16">
+        <v>89.1</v>
+      </c>
+      <c r="I100" s="17">
+        <v>0.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>